<commit_message>
Implementa estrutura inicial do histograma
</commit_message>
<xml_diff>
--- a/saida/F0009_000/Comparativo Cronograma 07-07-2026.xlsx
+++ b/saida/F0009_000/Comparativo Cronograma 07-07-2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bureauveritas.sharepoint.com/teams/POP-Planejamento/Shared Documents/Automacoes/Comparativo_Cronograma/saida/F0009_000/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="64" documentId="11_007A6A65FE3C53CA3EA3407FC89BECF8CCA5077D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5433D12C-E90E-4F0B-811D-B8CEB1CC1D34}"/>
+  <xr:revisionPtr revIDLastSave="76" documentId="11_007A6A65FE3C53CA3EA3407FC89BECF8CCA5077D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF2E4EEF-9853-4825-BA48-00755F2FEC18}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3317" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3300" uniqueCount="471">
   <si>
     <t>Id</t>
   </si>
@@ -1451,18 +1451,6 @@
     <t>COMP_AP</t>
   </si>
   <si>
-    <t>Soma</t>
-  </si>
-  <si>
-    <t>Média</t>
-  </si>
-  <si>
-    <t>Soma Acumulada</t>
-  </si>
-  <si>
-    <t>Contagem</t>
-  </si>
-  <si>
     <t>Coluna1</t>
   </si>
   <si>
@@ -1477,7 +1465,7 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1486,6 +1474,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1520,7 +1516,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1555,12 +1551,21 @@
     <xf numFmtId="9" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="151">
+  <dxfs count="164">
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1589,102 +1594,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1761,6 +1670,21 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1773,8 +1697,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1819,10 +1754,108 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1979,11 +2012,13 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2005,11 +2040,20 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -4055,7 +4099,7 @@
             <c:numRef>
               <c:f>'[1]Curva S'!$A$2:$A$120</c:f>
               <c:numCache>
-                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="119"/>
                 <c:pt idx="0">
                   <c:v>46101</c:v>
@@ -4817,7 +4861,7 @@
             <c:numRef>
               <c:f>'[1]Curva S'!$A$2:$A$120</c:f>
               <c:numCache>
-                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="119"/>
                 <c:pt idx="0">
                   <c:v>46101</c:v>
@@ -5599,7 +5643,7 @@
             <c:numRef>
               <c:f>'[1]Curva S'!$A$2:$A$120</c:f>
               <c:numCache>
-                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="119"/>
                 <c:pt idx="0">
                   <c:v>46101</c:v>
@@ -6376,7 +6420,7 @@
             <c:numRef>
               <c:f>'[1]Curva S'!$A$2:$A$120</c:f>
               <c:numCache>
-                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="119"/>
                 <c:pt idx="0">
                   <c:v>46101</c:v>
@@ -7094,14 +7138,14 @@
         <c:axId val="1737432527"/>
         <c:axId val="1737433007"/>
       </c:lineChart>
-      <c:dateAx>
+      <c:catAx>
         <c:axId val="1737432527"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="m/d/yyyy" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -7140,9 +7184,10 @@
         <c:crossAx val="1737433007"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:baseTimeUnit val="days"/>
-      </c:dateAx>
+        <c:noMultiLvlLbl val="1"/>
+      </c:catAx>
       <c:valAx>
         <c:axId val="1737433007"/>
         <c:scaling>
@@ -7239,23 +7284,24 @@
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
-      <c:dateAx>
+      <c:catAx>
         <c:axId val="1737439727"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="1"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="m/d/yyyy" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="1737437807"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:baseTimeUnit val="days"/>
-      </c:dateAx>
+        <c:noMultiLvlLbl val="1"/>
+      </c:catAx>
       <c:spPr>
         <a:noFill/>
         <a:ln>
@@ -7473,7 +7519,7 @@
             <c:numRef>
               <c:f>'[1]Curva S'!$A$2:$A$120</c:f>
               <c:numCache>
-                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="119"/>
                 <c:pt idx="0">
                   <c:v>46101</c:v>
@@ -8235,7 +8281,7 @@
             <c:numRef>
               <c:f>'[1]Curva S'!$A$2:$A$120</c:f>
               <c:numCache>
-                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="119"/>
                 <c:pt idx="0">
                   <c:v>46101</c:v>
@@ -8999,7 +9045,7 @@
             <c:numRef>
               <c:f>'[1]Curva S'!$A$2:$A$120</c:f>
               <c:numCache>
-                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="119"/>
                 <c:pt idx="0">
                   <c:v>46101</c:v>
@@ -9761,7 +9807,7 @@
             <c:numRef>
               <c:f>'[1]Curva S'!$A$2:$A$120</c:f>
               <c:numCache>
-                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="119"/>
                 <c:pt idx="0">
                   <c:v>46101</c:v>
@@ -10543,7 +10589,7 @@
             <c:numRef>
               <c:f>'[1]Curva S'!$A$2:$A$120</c:f>
               <c:numCache>
-                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="119"/>
                 <c:pt idx="0">
                   <c:v>46101</c:v>
@@ -11320,7 +11366,7 @@
             <c:numRef>
               <c:f>'[1]Curva S'!$A$2:$A$120</c:f>
               <c:numCache>
-                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="119"/>
                 <c:pt idx="0">
                   <c:v>46101</c:v>
@@ -12055,7 +12101,7 @@
             <c:numRef>
               <c:f>'[1]Curva S'!$A$2:$A$120</c:f>
               <c:numCache>
-                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="119"/>
                 <c:pt idx="0">
                   <c:v>46101</c:v>
@@ -12832,7 +12878,7 @@
             <c:numRef>
               <c:f>'[1]Curva S'!$A$2:$A$120</c:f>
               <c:numCache>
-                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="119"/>
                 <c:pt idx="0">
                   <c:v>46101</c:v>
@@ -13550,14 +13596,14 @@
         <c:axId val="1737386447"/>
         <c:axId val="1737387407"/>
       </c:lineChart>
-      <c:dateAx>
+      <c:catAx>
         <c:axId val="1737386447"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="m/d/yyyy" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -13596,9 +13642,10 @@
         <c:crossAx val="1737387407"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:baseTimeUnit val="days"/>
-      </c:dateAx>
+        <c:noMultiLvlLbl val="1"/>
+      </c:catAx>
       <c:valAx>
         <c:axId val="1737387407"/>
         <c:scaling>
@@ -13695,23 +13742,24 @@
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
-      <c:dateAx>
+      <c:catAx>
         <c:axId val="1737411407"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="1"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="m/d/yyyy" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="1737410447"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:baseTimeUnit val="days"/>
-      </c:dateAx>
+        <c:noMultiLvlLbl val="1"/>
+      </c:catAx>
       <c:spPr>
         <a:noFill/>
         <a:ln>
@@ -15058,561 +15106,7 @@
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
-      <sheetData sheetId="1">
-        <row r="3">
-          <cell r="B3" t="str">
-            <v>Emissão inicial total</v>
-          </cell>
-          <cell r="C3" t="str">
-            <v>Emissão inicial concluída</v>
-          </cell>
-          <cell r="D3" t="str">
-            <v>%EI</v>
-          </cell>
-          <cell r="E3" t="str">
-            <v>Avaliação do cliente concluída</v>
-          </cell>
-          <cell r="F3" t="str">
-            <v>Atendimento de comentário concluído</v>
-          </cell>
-          <cell r="G3" t="str">
-            <v>Aprovação concluída</v>
-          </cell>
-          <cell r="H3" t="str">
-            <v>%AP</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>AUTOMAÇÃO E INSTRUMENTAÇÃO</v>
-          </cell>
-          <cell r="B4">
-            <v>42</v>
-          </cell>
-          <cell r="C4">
-            <v>37</v>
-          </cell>
-          <cell r="D4">
-            <v>0.88095238095238093</v>
-          </cell>
-          <cell r="E4">
-            <v>3</v>
-          </cell>
-          <cell r="F4">
-            <v>0</v>
-          </cell>
-          <cell r="G4">
-            <v>0</v>
-          </cell>
-          <cell r="H4">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>CIVIL</v>
-          </cell>
-          <cell r="B5">
-            <v>2</v>
-          </cell>
-          <cell r="C5">
-            <v>0</v>
-          </cell>
-          <cell r="D5">
-            <v>0</v>
-          </cell>
-          <cell r="E5">
-            <v>0</v>
-          </cell>
-          <cell r="F5">
-            <v>0</v>
-          </cell>
-          <cell r="G5">
-            <v>0</v>
-          </cell>
-          <cell r="H5">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>COORDENAÇÃO</v>
-          </cell>
-          <cell r="B6">
-            <v>3</v>
-          </cell>
-          <cell r="C6">
-            <v>1</v>
-          </cell>
-          <cell r="D6">
-            <v>0.33333333333333331</v>
-          </cell>
-          <cell r="E6">
-            <v>1</v>
-          </cell>
-          <cell r="F6">
-            <v>0</v>
-          </cell>
-          <cell r="G6">
-            <v>0</v>
-          </cell>
-          <cell r="H6">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7" t="str">
-            <v>ELÉTRICA</v>
-          </cell>
-          <cell r="B7">
-            <v>3</v>
-          </cell>
-          <cell r="C7">
-            <v>3</v>
-          </cell>
-          <cell r="D7">
-            <v>1</v>
-          </cell>
-          <cell r="E7">
-            <v>2</v>
-          </cell>
-          <cell r="F7">
-            <v>0</v>
-          </cell>
-          <cell r="G7">
-            <v>0</v>
-          </cell>
-          <cell r="H7">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8" t="str">
-            <v>ESTRUTURA METÁLICA</v>
-          </cell>
-          <cell r="B8">
-            <v>14</v>
-          </cell>
-          <cell r="C8">
-            <v>0</v>
-          </cell>
-          <cell r="D8">
-            <v>0</v>
-          </cell>
-          <cell r="E8">
-            <v>0</v>
-          </cell>
-          <cell r="F8">
-            <v>0</v>
-          </cell>
-          <cell r="G8">
-            <v>0</v>
-          </cell>
-          <cell r="H8">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9" t="str">
-            <v>GERAL</v>
-          </cell>
-          <cell r="B9">
-            <v>0</v>
-          </cell>
-          <cell r="C9">
-            <v>0</v>
-          </cell>
-          <cell r="D9">
-            <v>0</v>
-          </cell>
-          <cell r="E9">
-            <v>0</v>
-          </cell>
-          <cell r="F9">
-            <v>0</v>
-          </cell>
-          <cell r="G9">
-            <v>0</v>
-          </cell>
-          <cell r="H9">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10" t="str">
-            <v>MARCOS</v>
-          </cell>
-          <cell r="B10">
-            <v>0</v>
-          </cell>
-          <cell r="C10">
-            <v>0</v>
-          </cell>
-          <cell r="D10">
-            <v>0</v>
-          </cell>
-          <cell r="E10">
-            <v>0</v>
-          </cell>
-          <cell r="F10">
-            <v>0</v>
-          </cell>
-          <cell r="G10">
-            <v>0</v>
-          </cell>
-          <cell r="H10">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11" t="str">
-            <v>MECÂNICA</v>
-          </cell>
-          <cell r="B11">
-            <v>25</v>
-          </cell>
-          <cell r="C11">
-            <v>16</v>
-          </cell>
-          <cell r="D11">
-            <v>0.64</v>
-          </cell>
-          <cell r="E11">
-            <v>4</v>
-          </cell>
-          <cell r="F11">
-            <v>1</v>
-          </cell>
-          <cell r="G11">
-            <v>1</v>
-          </cell>
-          <cell r="H11">
-            <v>0.04</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12" t="str">
-            <v>PENDÊNCIAS</v>
-          </cell>
-          <cell r="B12">
-            <v>0</v>
-          </cell>
-          <cell r="C12">
-            <v>0</v>
-          </cell>
-          <cell r="D12">
-            <v>0</v>
-          </cell>
-          <cell r="E12">
-            <v>0</v>
-          </cell>
-          <cell r="F12">
-            <v>0</v>
-          </cell>
-          <cell r="G12">
-            <v>0</v>
-          </cell>
-          <cell r="H12">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13" t="str">
-            <v>PLANEJAMENTO</v>
-          </cell>
-          <cell r="B13">
-            <v>2</v>
-          </cell>
-          <cell r="C13">
-            <v>2</v>
-          </cell>
-          <cell r="D13">
-            <v>1</v>
-          </cell>
-          <cell r="E13">
-            <v>2</v>
-          </cell>
-          <cell r="F13">
-            <v>2</v>
-          </cell>
-          <cell r="G13">
-            <v>2</v>
-          </cell>
-          <cell r="H13">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14" t="str">
-            <v>PROCESSOS</v>
-          </cell>
-          <cell r="B14">
-            <v>1</v>
-          </cell>
-          <cell r="C14">
-            <v>1</v>
-          </cell>
-          <cell r="D14">
-            <v>1</v>
-          </cell>
-          <cell r="E14">
-            <v>1</v>
-          </cell>
-          <cell r="F14">
-            <v>0</v>
-          </cell>
-          <cell r="G14">
-            <v>0</v>
-          </cell>
-          <cell r="H14">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="A15" t="str">
-            <v>TUBULAÇÃO / UTILIDADES</v>
-          </cell>
-          <cell r="B15">
-            <v>13</v>
-          </cell>
-          <cell r="C15">
-            <v>1</v>
-          </cell>
-          <cell r="D15">
-            <v>7.6923076923076927E-2</v>
-          </cell>
-          <cell r="E15">
-            <v>1</v>
-          </cell>
-          <cell r="F15">
-            <v>0</v>
-          </cell>
-          <cell r="G15">
-            <v>0</v>
-          </cell>
-          <cell r="H15">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="B21" t="str">
-            <v>Emissão Inicial Atrasada</v>
-          </cell>
-          <cell r="C21" t="str">
-            <v>Avaliação Cliente Atrasada</v>
-          </cell>
-          <cell r="D21" t="str">
-            <v>Atendimento Atrasado</v>
-          </cell>
-          <cell r="E21" t="str">
-            <v>Aprovação Atrasada</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="A22" t="str">
-            <v>AUTOMAÇÃO E INSTRUMENTAÇÃO</v>
-          </cell>
-          <cell r="B22">
-            <v>3</v>
-          </cell>
-          <cell r="C22">
-            <v>30</v>
-          </cell>
-          <cell r="D22">
-            <v>32</v>
-          </cell>
-          <cell r="E22">
-            <v>32</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="A23" t="str">
-            <v>CIVIL</v>
-          </cell>
-          <cell r="B23">
-            <v>0</v>
-          </cell>
-          <cell r="C23">
-            <v>0</v>
-          </cell>
-          <cell r="D23">
-            <v>0</v>
-          </cell>
-          <cell r="E23">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="A24" t="str">
-            <v>COORDENAÇÃO</v>
-          </cell>
-          <cell r="B24">
-            <v>1</v>
-          </cell>
-          <cell r="C24">
-            <v>0</v>
-          </cell>
-          <cell r="D24">
-            <v>0</v>
-          </cell>
-          <cell r="E24">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="A25" t="str">
-            <v>ELÉTRICA</v>
-          </cell>
-          <cell r="B25">
-            <v>0</v>
-          </cell>
-          <cell r="C25">
-            <v>0</v>
-          </cell>
-          <cell r="D25">
-            <v>2</v>
-          </cell>
-          <cell r="E25">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="26">
-          <cell r="A26" t="str">
-            <v>ESTRUTURA METÁLICA</v>
-          </cell>
-          <cell r="B26">
-            <v>0</v>
-          </cell>
-          <cell r="C26">
-            <v>0</v>
-          </cell>
-          <cell r="D26">
-            <v>0</v>
-          </cell>
-          <cell r="E26">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="27">
-          <cell r="A27" t="str">
-            <v>GERAL</v>
-          </cell>
-          <cell r="B27">
-            <v>0</v>
-          </cell>
-          <cell r="C27">
-            <v>0</v>
-          </cell>
-          <cell r="D27">
-            <v>0</v>
-          </cell>
-          <cell r="E27">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="28">
-          <cell r="A28" t="str">
-            <v>MARCOS</v>
-          </cell>
-          <cell r="B28">
-            <v>0</v>
-          </cell>
-          <cell r="C28">
-            <v>0</v>
-          </cell>
-          <cell r="D28">
-            <v>0</v>
-          </cell>
-          <cell r="E28">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="29">
-          <cell r="A29" t="str">
-            <v>MECÂNICA</v>
-          </cell>
-          <cell r="B29">
-            <v>1</v>
-          </cell>
-          <cell r="C29">
-            <v>11</v>
-          </cell>
-          <cell r="D29">
-            <v>14</v>
-          </cell>
-          <cell r="E29">
-            <v>8</v>
-          </cell>
-        </row>
-        <row r="30">
-          <cell r="A30" t="str">
-            <v>PENDÊNCIAS</v>
-          </cell>
-          <cell r="B30">
-            <v>0</v>
-          </cell>
-          <cell r="C30">
-            <v>0</v>
-          </cell>
-          <cell r="D30">
-            <v>0</v>
-          </cell>
-          <cell r="E30">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="A31" t="str">
-            <v>PLANEJAMENTO</v>
-          </cell>
-          <cell r="B31">
-            <v>0</v>
-          </cell>
-          <cell r="C31">
-            <v>0</v>
-          </cell>
-          <cell r="D31">
-            <v>0</v>
-          </cell>
-          <cell r="E31">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="32">
-          <cell r="A32" t="str">
-            <v>PROCESSOS</v>
-          </cell>
-          <cell r="B32">
-            <v>0</v>
-          </cell>
-          <cell r="C32">
-            <v>0</v>
-          </cell>
-          <cell r="D32">
-            <v>1</v>
-          </cell>
-          <cell r="E32">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="33">
-          <cell r="A33" t="str">
-            <v>TUBULAÇÃO / UTILIDADES</v>
-          </cell>
-          <cell r="B33">
-            <v>1</v>
-          </cell>
-          <cell r="C33">
-            <v>0</v>
-          </cell>
-          <cell r="D33">
-            <v>1</v>
-          </cell>
-          <cell r="E33">
-            <v>1</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="1"/>
       <sheetData sheetId="2">
         <row r="1">
           <cell r="B1" t="str">
@@ -19042,103 +18536,103 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{357AD549-C3E2-42CB-A5FF-BA8073049745}" name="Tabela3" displayName="Tabela3" ref="A1:AF184" totalsRowShown="0" headerRowDxfId="86" dataDxfId="85">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{357AD549-C3E2-42CB-A5FF-BA8073049745}" name="Tabela3" displayName="Tabela3" ref="A1:AF184" totalsRowShown="0" headerRowDxfId="129" dataDxfId="128">
   <autoFilter ref="A1:AF184" xr:uid="{357AD549-C3E2-42CB-A5FF-BA8073049745}"/>
   <tableColumns count="32">
-    <tableColumn id="1" xr3:uid="{105F9DB5-D3AE-463E-BEB6-B05A037292C1}" name="Id" dataDxfId="118"/>
-    <tableColumn id="2" xr3:uid="{FC0307A7-E14F-404E-BBD7-F1F9BA1F985B}" name="EDT" dataDxfId="117"/>
-    <tableColumn id="3" xr3:uid="{B6A8D4EA-92F5-472C-8A99-D66ABA8D3A16}" name="Nome do Resumo da Tarefa" dataDxfId="116"/>
-    <tableColumn id="4" xr3:uid="{350F8323-9B91-4129-A316-54FCEB05D2D1}" name="Nome da Tarefa" dataDxfId="115"/>
-    <tableColumn id="5" xr3:uid="{1FF55482-1749-4C26-A093-20CE4F6D5076}" name="Título" dataDxfId="114"/>
-    <tableColumn id="6" xr3:uid="{BE1B1D18-806D-467E-9289-F9586EAC00C5}" name="Duração" dataDxfId="113"/>
-    <tableColumn id="7" xr3:uid="{CAAC4D35-A840-4A7B-8353-CF3298C75AB6}" name="Início" dataDxfId="112"/>
-    <tableColumn id="8" xr3:uid="{84FFB9D2-C19D-4C61-A658-29309196A4D5}" name="Término" dataDxfId="111"/>
-    <tableColumn id="9" xr3:uid="{E67BDEA2-16FB-4A05-BE86-CF8F11528B87}" name="Predecessoras" dataDxfId="110"/>
-    <tableColumn id="10" xr3:uid="{5B2004D0-D8FB-4407-B788-AE1F87EA5A7B}" name="% concluída" dataDxfId="109" dataCellStyle="Porcentagem"/>
-    <tableColumn id="11" xr3:uid="{B6C9AFF1-D4A9-44AA-BF79-E0301A5CFB23}" name="Término real" dataDxfId="108"/>
-    <tableColumn id="12" xr3:uid="{BBD0501D-F2B3-4139-9F5F-07AC4A309DCB}" name="Status" dataDxfId="107"/>
-    <tableColumn id="13" xr3:uid="{AF84191D-890C-4A89-9106-76F2E134A24E}" name="Crítica" dataDxfId="106"/>
-    <tableColumn id="14" xr3:uid="{45DBC9FA-D781-4435-84F0-6B6381742796}" name="Disciplina" dataDxfId="105"/>
-    <tableColumn id="15" xr3:uid="{52232AA2-F80C-4ECF-8AF5-02CE4694F0A3}" name="Inicio_LB_R0" dataDxfId="104"/>
-    <tableColumn id="16" xr3:uid="{314E0FC3-A181-43AD-8926-20318FCB3730}" name="Término_LB_R0" dataDxfId="103"/>
-    <tableColumn id="17" xr3:uid="{700B5095-ED7E-4107-8EB8-DB535BBB734A}" name="Sprint" dataDxfId="102"/>
-    <tableColumn id="18" xr3:uid="{4257C684-F651-47FD-AF83-6801066B041F}" name="Sucessoras" dataDxfId="101"/>
-    <tableColumn id="19" xr3:uid="{2478AEDD-2887-47A9-B9CB-DEBE13A7EC68}" name="Comparação" dataDxfId="100"/>
-    <tableColumn id="20" xr3:uid="{694FD620-6B64-440E-B152-F102BB9982AF}" name="Nomes dos recursos" dataDxfId="99"/>
-    <tableColumn id="21" xr3:uid="{CDAFBC40-4A89-40C4-A78B-CC05513AA3E9}" name="pct_val" dataDxfId="98"/>
-    <tableColumn id="22" xr3:uid="{E2FF3321-7391-43C7-8544-5B66662A9CFA}" name="Emissão inicial total" dataDxfId="97"/>
-    <tableColumn id="23" xr3:uid="{0CBA4F68-2D06-45A1-8873-9ED5D342CBDA}" name="Emissão inicial concluída" dataDxfId="96"/>
-    <tableColumn id="24" xr3:uid="{B3526B9B-F566-4AB3-88E5-256E9B3EAD93}" name="Emissão Inicial Atrasada" dataDxfId="95"/>
-    <tableColumn id="25" xr3:uid="{73738602-87D2-4222-855A-C25F11326B62}" name="Aprovação total" dataDxfId="94"/>
-    <tableColumn id="26" xr3:uid="{8FA14EA7-E7B2-43E7-B81A-539428CFCF4C}" name="Avaliação do cliente concluída" dataDxfId="93"/>
-    <tableColumn id="27" xr3:uid="{62374080-8E23-41C3-AD80-FFC32A757A45}" name="Avaliação Cliente Atrasada" dataDxfId="92"/>
-    <tableColumn id="28" xr3:uid="{1B6732E8-5D2B-4F1C-81AA-A4664372F2B0}" name="Atendimento de comentário concluído" dataDxfId="91"/>
-    <tableColumn id="29" xr3:uid="{DCF558F7-5619-475E-8DEB-C2B0B75B1658}" name="Atendimento Atrasado" dataDxfId="90"/>
-    <tableColumn id="30" xr3:uid="{93C1D3A9-A2BF-4CA3-84F3-3E75E0C0A531}" name="Aprovação concluída" dataDxfId="89"/>
-    <tableColumn id="31" xr3:uid="{59DB34E2-BF46-419F-AEC7-E0DBBF0928B0}" name="Aprovação Atrasada" dataDxfId="88"/>
-    <tableColumn id="32" xr3:uid="{7FD7B756-D42D-42EA-B92C-9A3414A83209}" name="Aderência" dataDxfId="87"/>
+    <tableColumn id="1" xr3:uid="{105F9DB5-D3AE-463E-BEB6-B05A037292C1}" name="Id" dataDxfId="127"/>
+    <tableColumn id="2" xr3:uid="{FC0307A7-E14F-404E-BBD7-F1F9BA1F985B}" name="EDT" dataDxfId="126"/>
+    <tableColumn id="3" xr3:uid="{B6A8D4EA-92F5-472C-8A99-D66ABA8D3A16}" name="Nome do Resumo da Tarefa" dataDxfId="125"/>
+    <tableColumn id="4" xr3:uid="{350F8323-9B91-4129-A316-54FCEB05D2D1}" name="Nome da Tarefa" dataDxfId="124"/>
+    <tableColumn id="5" xr3:uid="{1FF55482-1749-4C26-A093-20CE4F6D5076}" name="Título" dataDxfId="123"/>
+    <tableColumn id="6" xr3:uid="{BE1B1D18-806D-467E-9289-F9586EAC00C5}" name="Duração" dataDxfId="122"/>
+    <tableColumn id="7" xr3:uid="{CAAC4D35-A840-4A7B-8353-CF3298C75AB6}" name="Início" dataDxfId="121"/>
+    <tableColumn id="8" xr3:uid="{84FFB9D2-C19D-4C61-A658-29309196A4D5}" name="Término" dataDxfId="120"/>
+    <tableColumn id="9" xr3:uid="{E67BDEA2-16FB-4A05-BE86-CF8F11528B87}" name="Predecessoras" dataDxfId="119"/>
+    <tableColumn id="10" xr3:uid="{5B2004D0-D8FB-4407-B788-AE1F87EA5A7B}" name="% concluída" dataDxfId="118" dataCellStyle="Porcentagem"/>
+    <tableColumn id="11" xr3:uid="{B6C9AFF1-D4A9-44AA-BF79-E0301A5CFB23}" name="Término real" dataDxfId="117"/>
+    <tableColumn id="12" xr3:uid="{BBD0501D-F2B3-4139-9F5F-07AC4A309DCB}" name="Status" dataDxfId="116"/>
+    <tableColumn id="13" xr3:uid="{AF84191D-890C-4A89-9106-76F2E134A24E}" name="Crítica" dataDxfId="115"/>
+    <tableColumn id="14" xr3:uid="{45DBC9FA-D781-4435-84F0-6B6381742796}" name="Disciplina" dataDxfId="114"/>
+    <tableColumn id="15" xr3:uid="{52232AA2-F80C-4ECF-8AF5-02CE4694F0A3}" name="Inicio_LB_R0" dataDxfId="113"/>
+    <tableColumn id="16" xr3:uid="{314E0FC3-A181-43AD-8926-20318FCB3730}" name="Término_LB_R0" dataDxfId="112"/>
+    <tableColumn id="17" xr3:uid="{700B5095-ED7E-4107-8EB8-DB535BBB734A}" name="Sprint" dataDxfId="111"/>
+    <tableColumn id="18" xr3:uid="{4257C684-F651-47FD-AF83-6801066B041F}" name="Sucessoras" dataDxfId="110"/>
+    <tableColumn id="19" xr3:uid="{2478AEDD-2887-47A9-B9CB-DEBE13A7EC68}" name="Comparação" dataDxfId="109"/>
+    <tableColumn id="20" xr3:uid="{694FD620-6B64-440E-B152-F102BB9982AF}" name="Nomes dos recursos" dataDxfId="108"/>
+    <tableColumn id="21" xr3:uid="{CDAFBC40-4A89-40C4-A78B-CC05513AA3E9}" name="pct_val" dataDxfId="107"/>
+    <tableColumn id="22" xr3:uid="{E2FF3321-7391-43C7-8544-5B66662A9CFA}" name="Emissão inicial total" dataDxfId="106"/>
+    <tableColumn id="23" xr3:uid="{0CBA4F68-2D06-45A1-8873-9ED5D342CBDA}" name="Emissão inicial concluída" dataDxfId="105"/>
+    <tableColumn id="24" xr3:uid="{B3526B9B-F566-4AB3-88E5-256E9B3EAD93}" name="Emissão Inicial Atrasada" dataDxfId="104"/>
+    <tableColumn id="25" xr3:uid="{73738602-87D2-4222-855A-C25F11326B62}" name="Aprovação total" dataDxfId="103"/>
+    <tableColumn id="26" xr3:uid="{8FA14EA7-E7B2-43E7-B81A-539428CFCF4C}" name="Avaliação do cliente concluída" dataDxfId="102"/>
+    <tableColumn id="27" xr3:uid="{62374080-8E23-41C3-AD80-FFC32A757A45}" name="Avaliação Cliente Atrasada" dataDxfId="101"/>
+    <tableColumn id="28" xr3:uid="{1B6732E8-5D2B-4F1C-81AA-A4664372F2B0}" name="Atendimento de comentário concluído" dataDxfId="100"/>
+    <tableColumn id="29" xr3:uid="{DCF558F7-5619-475E-8DEB-C2B0B75B1658}" name="Atendimento Atrasado" dataDxfId="99"/>
+    <tableColumn id="30" xr3:uid="{93C1D3A9-A2BF-4CA3-84F3-3E75E0C0A531}" name="Aprovação concluída" dataDxfId="98"/>
+    <tableColumn id="31" xr3:uid="{59DB34E2-BF46-419F-AEC7-E0DBBF0928B0}" name="Aprovação Atrasada" dataDxfId="97"/>
+    <tableColumn id="32" xr3:uid="{7FD7B756-D42D-42EA-B92C-9A3414A83209}" name="Aderência" dataDxfId="96"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6AF6E3E3-4F0C-4448-8ABB-84C816C7E55F}" name="Tabela1" displayName="Tabela1" ref="A3:H17" totalsRowCount="1" headerRowDxfId="134" dataDxfId="132" totalsRowDxfId="133">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6AF6E3E3-4F0C-4448-8ABB-84C816C7E55F}" name="Tabela1" displayName="Tabela1" ref="A3:H17" totalsRowCount="1" headerRowDxfId="95" dataDxfId="94" totalsRowDxfId="93">
   <autoFilter ref="A3:H16" xr:uid="{6AF6E3E3-4F0C-4448-8ABB-84C816C7E55F}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{02F46B2B-A028-47E2-96FA-2276CD1E109B}" name="Disciplina" totalsRowLabel="TOTAL" dataDxfId="150" totalsRowDxfId="149"/>
-    <tableColumn id="2" xr3:uid="{73EFD3B7-B098-4A11-BEDA-C08ABFB8DB05}" name="Emissão inicial total" totalsRowFunction="sum" dataDxfId="148" totalsRowDxfId="147"/>
-    <tableColumn id="3" xr3:uid="{7C14357F-B9C2-418E-A7F2-EB1748D0A9F2}" name="Emissão inicial concluída" totalsRowFunction="sum" dataDxfId="146" totalsRowDxfId="145"/>
-    <tableColumn id="4" xr3:uid="{3F5AF0A6-D562-43AD-B14A-073760C3EEA7}" name="%EI" dataDxfId="144" totalsRowDxfId="143"/>
-    <tableColumn id="5" xr3:uid="{9BA1141B-D47D-4151-83D2-8C32EBDEEB25}" name="Avaliação do cliente concluída" totalsRowFunction="sum" dataDxfId="142" totalsRowDxfId="141"/>
-    <tableColumn id="6" xr3:uid="{C5BFCC78-8F26-485B-BB31-666C5727FB48}" name="Atendimento de comentário concluído" totalsRowFunction="sum" dataDxfId="140" totalsRowDxfId="139"/>
-    <tableColumn id="7" xr3:uid="{D0B8BD1F-2690-4EDF-9681-E40C394EAA0D}" name="Aprovação concluída" totalsRowFunction="sum" dataDxfId="138" totalsRowDxfId="137"/>
-    <tableColumn id="8" xr3:uid="{C9D6CADA-9664-46F7-983E-D4CAFCCD4BA2}" name="%AP" dataDxfId="136" totalsRowDxfId="135"/>
+    <tableColumn id="1" xr3:uid="{02F46B2B-A028-47E2-96FA-2276CD1E109B}" name="Disciplina" totalsRowLabel="TOTAL" dataDxfId="92" totalsRowDxfId="91"/>
+    <tableColumn id="2" xr3:uid="{73EFD3B7-B098-4A11-BEDA-C08ABFB8DB05}" name="Emissão inicial total" totalsRowFunction="sum" dataDxfId="90" totalsRowDxfId="89"/>
+    <tableColumn id="3" xr3:uid="{7C14357F-B9C2-418E-A7F2-EB1748D0A9F2}" name="Emissão inicial concluída" totalsRowFunction="sum" dataDxfId="88" totalsRowDxfId="87"/>
+    <tableColumn id="4" xr3:uid="{3F5AF0A6-D562-43AD-B14A-073760C3EEA7}" name="%EI" dataDxfId="86" totalsRowDxfId="85"/>
+    <tableColumn id="5" xr3:uid="{9BA1141B-D47D-4151-83D2-8C32EBDEEB25}" name="Avaliação do cliente concluída" totalsRowFunction="sum" dataDxfId="84" totalsRowDxfId="83"/>
+    <tableColumn id="6" xr3:uid="{C5BFCC78-8F26-485B-BB31-666C5727FB48}" name="Atendimento de comentário concluído" totalsRowFunction="sum" dataDxfId="82" totalsRowDxfId="81"/>
+    <tableColumn id="7" xr3:uid="{D0B8BD1F-2690-4EDF-9681-E40C394EAA0D}" name="Aprovação concluída" totalsRowFunction="sum" dataDxfId="80" totalsRowDxfId="79"/>
+    <tableColumn id="8" xr3:uid="{C9D6CADA-9664-46F7-983E-D4CAFCCD4BA2}" name="%AP" dataDxfId="78" totalsRowDxfId="77"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E423278C-188B-4480-B6D9-8EDE6CCEB649}" name="Tabela2" displayName="Tabela2" ref="A22:E36" totalsRowCount="1" headerRowDxfId="121" dataDxfId="119" totalsRowDxfId="120">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E423278C-188B-4480-B6D9-8EDE6CCEB649}" name="Tabela2" displayName="Tabela2" ref="A22:E36" totalsRowCount="1" headerRowDxfId="76" dataDxfId="75" totalsRowDxfId="74">
   <autoFilter ref="A22:E35" xr:uid="{E423278C-188B-4480-B6D9-8EDE6CCEB649}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{E8C29044-3E28-4511-BAEF-827EFCA81D0D}" name="Disciplina" totalsRowLabel="TOTAL" dataDxfId="131" totalsRowDxfId="130"/>
-    <tableColumn id="2" xr3:uid="{29DF3239-3D2C-435C-BC95-223D9C37B34D}" name="Emissão Inicial Atrasada" totalsRowFunction="sum" dataDxfId="129" totalsRowDxfId="128"/>
-    <tableColumn id="3" xr3:uid="{234A0119-8A2F-4536-B8A7-C185A0E7356E}" name="Avaliação Cliente Atrasada" totalsRowFunction="sum" dataDxfId="127" totalsRowDxfId="126"/>
-    <tableColumn id="4" xr3:uid="{9A3B27A8-5632-465B-9C00-3F7EFF2C4130}" name="Atendimento Atrasado" totalsRowFunction="sum" dataDxfId="125" totalsRowDxfId="124"/>
-    <tableColumn id="5" xr3:uid="{92CABBF9-FB8E-49FD-A68B-31D5AC76B130}" name="Aprovação Atrasada" totalsRowFunction="sum" dataDxfId="123" totalsRowDxfId="122"/>
+    <tableColumn id="1" xr3:uid="{E8C29044-3E28-4511-BAEF-827EFCA81D0D}" name="Disciplina" totalsRowLabel="TOTAL" dataDxfId="73" totalsRowDxfId="72"/>
+    <tableColumn id="2" xr3:uid="{29DF3239-3D2C-435C-BC95-223D9C37B34D}" name="Emissão Inicial Atrasada" totalsRowFunction="sum" dataDxfId="71" totalsRowDxfId="70"/>
+    <tableColumn id="3" xr3:uid="{234A0119-8A2F-4536-B8A7-C185A0E7356E}" name="Avaliação Cliente Atrasada" totalsRowFunction="sum" dataDxfId="69" totalsRowDxfId="68"/>
+    <tableColumn id="4" xr3:uid="{9A3B27A8-5632-465B-9C00-3F7EFF2C4130}" name="Atendimento Atrasado" totalsRowFunction="sum" dataDxfId="67" totalsRowDxfId="66"/>
+    <tableColumn id="5" xr3:uid="{92CABBF9-FB8E-49FD-A68B-31D5AC76B130}" name="Aprovação Atrasada" totalsRowFunction="sum" dataDxfId="65" totalsRowDxfId="64"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A92AC415-BAD4-4F0E-9672-62E6F796897D}" name="Tabela4" displayName="Tabela4" ref="A1:O183" totalsRowShown="0" headerRowDxfId="71" dataDxfId="70">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A92AC415-BAD4-4F0E-9672-62E6F796897D}" name="Tabela4" displayName="Tabela4" ref="A1:O183" totalsRowShown="0" headerRowDxfId="63" dataDxfId="62">
   <autoFilter ref="A1:O183" xr:uid="{A92AC415-BAD4-4F0E-9672-62E6F796897D}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{9AA0EEEC-3DDA-4059-8C2B-0639FC8B63E2}" name="Data" dataDxfId="68"/>
-    <tableColumn id="2" xr3:uid="{AD507717-4CBE-4C5F-BF83-180325A49DEF}" name="Emissão prevista na LB" dataDxfId="69"/>
-    <tableColumn id="3" xr3:uid="{DF69B074-EBF0-4027-A234-269EDDAD7464}" name="Emissão prevista na LB acumulada" dataDxfId="84"/>
-    <tableColumn id="4" xr3:uid="{7243D4A6-BF9B-4477-A29B-BBE6907AA4FB}" name="Emissão realizada por dia" dataDxfId="83"/>
-    <tableColumn id="5" xr3:uid="{16E43178-ADC6-42D4-B6FA-49A77E660B35}" name="Emissão realizada acumulada" dataDxfId="82"/>
-    <tableColumn id="6" xr3:uid="{8AF62C70-AC94-4913-BCEC-22038B232985}" name="Aprovação prevista na LB" dataDxfId="81"/>
-    <tableColumn id="7" xr3:uid="{9573BF78-042E-46A1-BB5D-5F19B075E258}" name="Aprovação realizada por dia" dataDxfId="80"/>
-    <tableColumn id="8" xr3:uid="{1A061C2F-F8BB-4D8C-AFD7-D47395971083}" name="Aprovação prevista na LB acumulada" dataDxfId="79"/>
-    <tableColumn id="9" xr3:uid="{D08189EC-CFFE-4445-AB1F-25ADD009B2C3}" name="Aprovação realizada acumulada" dataDxfId="78"/>
-    <tableColumn id="10" xr3:uid="{CF7F8CB1-CB02-4ADC-99D6-A5CF977984D4}" name="Avanço da EI previsto na LB" dataDxfId="77" dataCellStyle="Porcentagem"/>
-    <tableColumn id="11" xr3:uid="{B75F05C3-2707-4825-AE52-AE96E576BA7B}" name="Avanço real da EI na LB" dataDxfId="76" dataCellStyle="Porcentagem"/>
-    <tableColumn id="12" xr3:uid="{325E4CB5-C75A-40A2-906B-F8763CBA509C}" name="COMP_EI" dataDxfId="75"/>
-    <tableColumn id="13" xr3:uid="{34960980-3580-43C6-B438-AEEFB1DDF412}" name="Avanço da AP previsto na LB" dataDxfId="74" dataCellStyle="Porcentagem"/>
-    <tableColumn id="14" xr3:uid="{1C71F75E-62B1-4D99-B699-9475192AD5C4}" name="Avanço da AP real na LB" dataDxfId="73" dataCellStyle="Porcentagem"/>
-    <tableColumn id="15" xr3:uid="{6CBEF4E1-83EF-4DD3-A005-E43F9D3E55D7}" name="COMP_AP" dataDxfId="72"/>
+    <tableColumn id="1" xr3:uid="{9AA0EEEC-3DDA-4059-8C2B-0639FC8B63E2}" name="Data" dataDxfId="61"/>
+    <tableColumn id="2" xr3:uid="{AD507717-4CBE-4C5F-BF83-180325A49DEF}" name="Emissão prevista na LB" dataDxfId="60"/>
+    <tableColumn id="3" xr3:uid="{DF69B074-EBF0-4027-A234-269EDDAD7464}" name="Emissão prevista na LB acumulada" dataDxfId="59"/>
+    <tableColumn id="4" xr3:uid="{7243D4A6-BF9B-4477-A29B-BBE6907AA4FB}" name="Emissão realizada por dia" dataDxfId="58"/>
+    <tableColumn id="5" xr3:uid="{16E43178-ADC6-42D4-B6FA-49A77E660B35}" name="Emissão realizada acumulada" dataDxfId="57"/>
+    <tableColumn id="6" xr3:uid="{8AF62C70-AC94-4913-BCEC-22038B232985}" name="Aprovação prevista na LB" dataDxfId="56"/>
+    <tableColumn id="7" xr3:uid="{9573BF78-042E-46A1-BB5D-5F19B075E258}" name="Aprovação realizada por dia" dataDxfId="55"/>
+    <tableColumn id="8" xr3:uid="{1A061C2F-F8BB-4D8C-AFD7-D47395971083}" name="Aprovação prevista na LB acumulada" dataDxfId="54"/>
+    <tableColumn id="9" xr3:uid="{D08189EC-CFFE-4445-AB1F-25ADD009B2C3}" name="Aprovação realizada acumulada" dataDxfId="53"/>
+    <tableColumn id="10" xr3:uid="{CF7F8CB1-CB02-4ADC-99D6-A5CF977984D4}" name="Avanço da EI previsto na LB" dataDxfId="52" dataCellStyle="Porcentagem"/>
+    <tableColumn id="11" xr3:uid="{B75F05C3-2707-4825-AE52-AE96E576BA7B}" name="Avanço real da EI na LB" dataDxfId="51" dataCellStyle="Porcentagem"/>
+    <tableColumn id="12" xr3:uid="{325E4CB5-C75A-40A2-906B-F8763CBA509C}" name="COMP_EI" dataDxfId="50"/>
+    <tableColumn id="13" xr3:uid="{34960980-3580-43C6-B438-AEEFB1DDF412}" name="Avanço da AP previsto na LB" dataDxfId="49" dataCellStyle="Porcentagem"/>
+    <tableColumn id="14" xr3:uid="{1C71F75E-62B1-4D99-B699-9475192AD5C4}" name="Avanço da AP real na LB" dataDxfId="48" dataCellStyle="Porcentagem"/>
+    <tableColumn id="15" xr3:uid="{6CBEF4E1-83EF-4DD3-A005-E43F9D3E55D7}" name="COMP_AP" dataDxfId="47"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{8F967D62-5B9F-437A-B655-135D5A3C5C1E}" name="Tabela5" displayName="Tabela5" ref="A1:AF31" totalsRowShown="0" headerRowDxfId="42" dataDxfId="41">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{8F967D62-5B9F-437A-B655-135D5A3C5C1E}" name="Tabela5" displayName="Tabela5" ref="A1:AF31" totalsRowShown="0" headerRowDxfId="46" dataDxfId="45">
   <autoFilter ref="A1:AF31" xr:uid="{8F967D62-5B9F-437A-B655-135D5A3C5C1E}">
     <filterColumn colId="3">
       <filters>
@@ -19147,45 +18641,45 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="32">
-    <tableColumn id="1" xr3:uid="{C358C923-D9DA-4B18-A238-A23EDB10D746}" name="Id" dataDxfId="67"/>
-    <tableColumn id="2" xr3:uid="{22631AA6-96C7-4C4F-A61B-FA2B853D79C0}" name="EDT" dataDxfId="66"/>
-    <tableColumn id="3" xr3:uid="{2BE4E7BF-35AF-4370-B406-3839A015AA12}" name="Nome do Resumo da Tarefa" dataDxfId="65"/>
-    <tableColumn id="4" xr3:uid="{14B1D489-0414-44B6-A9A5-31FACF1C2FF2}" name="Nome da Tarefa" dataDxfId="64"/>
-    <tableColumn id="5" xr3:uid="{233E069F-7B7D-4EF5-9F06-7D54E507C760}" name="Título" dataDxfId="63"/>
-    <tableColumn id="6" xr3:uid="{065DDDE4-D0A2-4987-A84E-F8AEA8BE3300}" name="Duração" dataDxfId="40"/>
-    <tableColumn id="7" xr3:uid="{BF551C86-B435-443C-A0E9-29BD0212FD0E}" name="Início" dataDxfId="39"/>
+    <tableColumn id="1" xr3:uid="{C358C923-D9DA-4B18-A238-A23EDB10D746}" name="Id" dataDxfId="44"/>
+    <tableColumn id="2" xr3:uid="{22631AA6-96C7-4C4F-A61B-FA2B853D79C0}" name="EDT" dataDxfId="43"/>
+    <tableColumn id="3" xr3:uid="{2BE4E7BF-35AF-4370-B406-3839A015AA12}" name="Nome do Resumo da Tarefa" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{14B1D489-0414-44B6-A9A5-31FACF1C2FF2}" name="Nome da Tarefa" dataDxfId="41"/>
+    <tableColumn id="5" xr3:uid="{233E069F-7B7D-4EF5-9F06-7D54E507C760}" name="Título" dataDxfId="40"/>
+    <tableColumn id="6" xr3:uid="{065DDDE4-D0A2-4987-A84E-F8AEA8BE3300}" name="Duração" dataDxfId="39"/>
+    <tableColumn id="7" xr3:uid="{BF551C86-B435-443C-A0E9-29BD0212FD0E}" name="Início" dataDxfId="38"/>
     <tableColumn id="8" xr3:uid="{CF69C541-43CD-4104-86CF-F541D39CDD59}" name="Término" dataDxfId="37"/>
-    <tableColumn id="9" xr3:uid="{D999710A-D4BC-4C7B-A09A-D1A884B4C8E6}" name="Predecessoras" dataDxfId="38"/>
-    <tableColumn id="10" xr3:uid="{408001A8-0463-4587-ADC6-D79C44F3B67F}" name="% concluída" dataDxfId="36" dataCellStyle="Porcentagem"/>
+    <tableColumn id="9" xr3:uid="{D999710A-D4BC-4C7B-A09A-D1A884B4C8E6}" name="Predecessoras" dataDxfId="36"/>
+    <tableColumn id="10" xr3:uid="{408001A8-0463-4587-ADC6-D79C44F3B67F}" name="% concluída" dataDxfId="35" dataCellStyle="Porcentagem"/>
     <tableColumn id="11" xr3:uid="{CFB0DC0C-2B25-4F7A-89DD-3ECEB8880AD1}" name="Término real" dataDxfId="34"/>
-    <tableColumn id="12" xr3:uid="{6D841E01-72EA-4490-8A0E-2CB9587CBBA6}" name="Status" dataDxfId="35"/>
-    <tableColumn id="13" xr3:uid="{C4B3E738-0DE8-4BED-AE87-C768933C9279}" name="Crítica" dataDxfId="62"/>
-    <tableColumn id="14" xr3:uid="{9DEB7B1A-13BE-4703-8085-6BA8112E5194}" name="Disciplina" dataDxfId="61"/>
-    <tableColumn id="15" xr3:uid="{9789D46F-BF83-4657-A82D-A4D40F74F80C}" name="Inicio_LB_R0" dataDxfId="60"/>
-    <tableColumn id="16" xr3:uid="{6404286C-FA52-4A76-9F30-355D9DE5DAF7}" name="Término_LB_R0" dataDxfId="59"/>
-    <tableColumn id="17" xr3:uid="{B1389D9D-8D9A-42D2-A270-A71EC49F0360}" name="Sprint" dataDxfId="58"/>
-    <tableColumn id="18" xr3:uid="{A8DAF246-9A19-45C7-BAEB-109970F000C3}" name="Sucessoras" dataDxfId="57"/>
-    <tableColumn id="19" xr3:uid="{C8ED20DC-CD8D-4038-BAF4-33B0729E362D}" name="Comparação" dataDxfId="56"/>
-    <tableColumn id="20" xr3:uid="{28A1EE4D-9D39-4B28-AF20-23E3EB1597C3}" name="Nomes dos recursos" dataDxfId="55"/>
-    <tableColumn id="21" xr3:uid="{D40F5EE6-8904-4657-A3B3-7122129F98E1}" name="pct_val" dataDxfId="54"/>
-    <tableColumn id="22" xr3:uid="{C495ADD0-B27F-4CDF-B40C-9D3C20C3550C}" name="Emissão inicial total" dataDxfId="53"/>
-    <tableColumn id="23" xr3:uid="{0FCD2336-1247-402B-AE01-F04463BBEC19}" name="Emissão inicial concluída" dataDxfId="52"/>
-    <tableColumn id="24" xr3:uid="{2CF9F0BF-3282-47D9-A524-45DC6857FAE9}" name="Emissão Inicial Atrasada" dataDxfId="51"/>
-    <tableColumn id="25" xr3:uid="{A4189055-AF46-4FE5-B59C-E8DF7447AF26}" name="Aprovação total" dataDxfId="50"/>
-    <tableColumn id="26" xr3:uid="{B3EFEFBD-DD11-4D3C-922E-98EE9E823681}" name="Avaliação do cliente concluída" dataDxfId="49"/>
-    <tableColumn id="27" xr3:uid="{EF88031B-07A2-4268-AB01-9B13F09541DC}" name="Avaliação Cliente Atrasada" dataDxfId="48"/>
-    <tableColumn id="28" xr3:uid="{C6038F68-7992-46CF-B1E9-210A49E90B08}" name="Atendimento de comentário concluído" dataDxfId="47"/>
-    <tableColumn id="29" xr3:uid="{B7217DEE-6A7A-47F6-81EC-8E6FED6CFD96}" name="Atendimento Atrasado" dataDxfId="46"/>
-    <tableColumn id="30" xr3:uid="{E77C0C95-5766-4F08-9A63-AA23BD30A387}" name="Aprovação concluída" dataDxfId="45"/>
-    <tableColumn id="31" xr3:uid="{BCBDEB55-ED60-4800-934B-15C01F761D98}" name="Aprovação Atrasada" dataDxfId="44"/>
-    <tableColumn id="32" xr3:uid="{F87511C8-1D54-4410-8800-1A4A44A2512B}" name="Aderência" dataDxfId="43"/>
+    <tableColumn id="12" xr3:uid="{6D841E01-72EA-4490-8A0E-2CB9587CBBA6}" name="Status" dataDxfId="33"/>
+    <tableColumn id="13" xr3:uid="{C4B3E738-0DE8-4BED-AE87-C768933C9279}" name="Crítica" dataDxfId="32"/>
+    <tableColumn id="14" xr3:uid="{9DEB7B1A-13BE-4703-8085-6BA8112E5194}" name="Disciplina" dataDxfId="31"/>
+    <tableColumn id="15" xr3:uid="{9789D46F-BF83-4657-A82D-A4D40F74F80C}" name="Inicio_LB_R0" dataDxfId="30"/>
+    <tableColumn id="16" xr3:uid="{6404286C-FA52-4A76-9F30-355D9DE5DAF7}" name="Término_LB_R0" dataDxfId="29"/>
+    <tableColumn id="17" xr3:uid="{B1389D9D-8D9A-42D2-A270-A71EC49F0360}" name="Sprint" dataDxfId="28"/>
+    <tableColumn id="18" xr3:uid="{A8DAF246-9A19-45C7-BAEB-109970F000C3}" name="Sucessoras" dataDxfId="27"/>
+    <tableColumn id="19" xr3:uid="{C8ED20DC-CD8D-4038-BAF4-33B0729E362D}" name="Comparação" dataDxfId="26"/>
+    <tableColumn id="20" xr3:uid="{28A1EE4D-9D39-4B28-AF20-23E3EB1597C3}" name="Nomes dos recursos" dataDxfId="25"/>
+    <tableColumn id="21" xr3:uid="{D40F5EE6-8904-4657-A3B3-7122129F98E1}" name="pct_val" dataDxfId="24"/>
+    <tableColumn id="22" xr3:uid="{C495ADD0-B27F-4CDF-B40C-9D3C20C3550C}" name="Emissão inicial total" dataDxfId="23"/>
+    <tableColumn id="23" xr3:uid="{0FCD2336-1247-402B-AE01-F04463BBEC19}" name="Emissão inicial concluída" dataDxfId="22"/>
+    <tableColumn id="24" xr3:uid="{2CF9F0BF-3282-47D9-A524-45DC6857FAE9}" name="Emissão Inicial Atrasada" dataDxfId="21"/>
+    <tableColumn id="25" xr3:uid="{A4189055-AF46-4FE5-B59C-E8DF7447AF26}" name="Aprovação total" dataDxfId="20"/>
+    <tableColumn id="26" xr3:uid="{B3EFEFBD-DD11-4D3C-922E-98EE9E823681}" name="Avaliação do cliente concluída" dataDxfId="19"/>
+    <tableColumn id="27" xr3:uid="{EF88031B-07A2-4268-AB01-9B13F09541DC}" name="Avaliação Cliente Atrasada" dataDxfId="18"/>
+    <tableColumn id="28" xr3:uid="{C6038F68-7992-46CF-B1E9-210A49E90B08}" name="Atendimento de comentário concluído" dataDxfId="17"/>
+    <tableColumn id="29" xr3:uid="{B7217DEE-6A7A-47F6-81EC-8E6FED6CFD96}" name="Atendimento Atrasado" dataDxfId="16"/>
+    <tableColumn id="30" xr3:uid="{E77C0C95-5766-4F08-9A63-AA23BD30A387}" name="Aprovação concluída" dataDxfId="15"/>
+    <tableColumn id="31" xr3:uid="{BCBDEB55-ED60-4800-934B-15C01F761D98}" name="Aprovação Atrasada" dataDxfId="14"/>
+    <tableColumn id="32" xr3:uid="{F87511C8-1D54-4410-8800-1A4A44A2512B}" name="Aderência" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{20E9742C-4A9D-462F-9710-931030E25F8B}" name="Tabela6" displayName="Tabela6" ref="A1:AF50" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{20E9742C-4A9D-462F-9710-931030E25F8B}" name="Tabela6" displayName="Tabela6" ref="A1:AF50" totalsRowShown="0" headerRowDxfId="163" dataDxfId="162">
   <autoFilter ref="A1:AF50" xr:uid="{20E9742C-4A9D-462F-9710-931030E25F8B}">
     <filterColumn colId="3">
       <filters>
@@ -19194,38 +18688,64 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="32">
-    <tableColumn id="1" xr3:uid="{32358809-4D84-4EC6-9D6B-F35560F3DC76}" name="Id" dataDxfId="33"/>
-    <tableColumn id="2" xr3:uid="{FCB19FCF-87B1-4F17-A0AF-E2A9C7A37E14}" name="EDT" dataDxfId="32"/>
-    <tableColumn id="3" xr3:uid="{7B4C3492-A62F-4D65-BBF2-069B72009597}" name="Nome do Resumo da Tarefa" dataDxfId="31"/>
-    <tableColumn id="4" xr3:uid="{AD7B3DE1-9E98-459C-BDE3-9919792FF211}" name="Nome da Tarefa" dataDxfId="30"/>
-    <tableColumn id="5" xr3:uid="{92DFDBD7-E2BA-4076-951E-CF16C7ACC9C8}" name="Título" dataDxfId="29"/>
-    <tableColumn id="6" xr3:uid="{AC61FD1A-02A4-4608-AD57-A107FA721510}" name="Duração" dataDxfId="28"/>
-    <tableColumn id="7" xr3:uid="{9BE80CD5-26B0-4EB9-A979-0FC73B0DA5C1}" name="Início" dataDxfId="27"/>
-    <tableColumn id="8" xr3:uid="{C042A1D2-CD11-451A-BB2E-ADF748E717B7}" name="Término" dataDxfId="26"/>
-    <tableColumn id="9" xr3:uid="{34B72A3E-C902-4F09-A15E-BE98CDEBA5DC}" name="Predecessoras" dataDxfId="25"/>
-    <tableColumn id="10" xr3:uid="{31D2A1DA-CB2D-4FF9-804B-2BCF79701600}" name="% concluída" dataDxfId="24"/>
-    <tableColumn id="11" xr3:uid="{1C5DB045-C98A-41DA-A131-D34F37499306}" name="Término real" dataDxfId="23"/>
-    <tableColumn id="12" xr3:uid="{C5DBA407-4507-4B9D-A13E-CF0E5B37F4CB}" name="Status" dataDxfId="22"/>
-    <tableColumn id="13" xr3:uid="{7FD0F52D-F14B-4094-9B86-E31407658E6F}" name="Crítica" dataDxfId="21"/>
-    <tableColumn id="14" xr3:uid="{7C23A16E-8B3B-4CE8-AC03-22AC7CF72944}" name="Disciplina" dataDxfId="20"/>
-    <tableColumn id="15" xr3:uid="{88A23DF0-3034-4C7F-88CF-2DB38B1912FA}" name="Inicio_LB_R0" dataDxfId="19"/>
-    <tableColumn id="16" xr3:uid="{392A346F-3130-451B-A21F-E3796E7334D3}" name="Término_LB_R0" dataDxfId="18"/>
-    <tableColumn id="17" xr3:uid="{B9376082-58D3-49C9-A5B2-3C92CDBDEF3F}" name="Sprint" dataDxfId="17"/>
-    <tableColumn id="18" xr3:uid="{0CF4B4D4-ADC5-4588-B459-CC9363BB628A}" name="Sucessoras" dataDxfId="16"/>
-    <tableColumn id="19" xr3:uid="{DC3CD69F-D143-4C72-A08D-3F6B3D9E2249}" name="Comparação" dataDxfId="15"/>
-    <tableColumn id="20" xr3:uid="{945E3C0B-F472-404B-908F-FA76314CBA06}" name="Nomes dos recursos" dataDxfId="14"/>
-    <tableColumn id="21" xr3:uid="{E8B58DDB-65B5-4CA3-BC94-BC6B83061F33}" name="pct_val" dataDxfId="13"/>
-    <tableColumn id="22" xr3:uid="{082E8DFC-12B4-4EF3-BF47-3B3E6C3402E6}" name="Emissão inicial total" dataDxfId="12"/>
-    <tableColumn id="23" xr3:uid="{56C00BFF-1CD0-4CA8-84E4-E64001C6BED1}" name="Emissão inicial concluída" dataDxfId="11"/>
-    <tableColumn id="24" xr3:uid="{D2BA410D-4E72-405E-8AE7-050A5615443E}" name="Emissão Inicial Atrasada" dataDxfId="10"/>
-    <tableColumn id="25" xr3:uid="{675921B6-37F4-4A25-8D73-49B885233FFB}" name="Aprovação total" dataDxfId="9"/>
-    <tableColumn id="26" xr3:uid="{EACBFD06-8091-40A3-84B2-A054E3939CBE}" name="Avaliação do cliente concluída" dataDxfId="8"/>
-    <tableColumn id="27" xr3:uid="{FB495C50-A60D-4AA1-993F-9434537E0198}" name="Avaliação Cliente Atrasada" dataDxfId="7"/>
-    <tableColumn id="28" xr3:uid="{A73FCDFE-A256-4469-830F-FEED2901F101}" name="Atendimento de comentário concluído" dataDxfId="6"/>
-    <tableColumn id="29" xr3:uid="{79F7235A-C25E-4E99-8A10-F9E041C573F8}" name="Atendimento Atrasado" dataDxfId="5"/>
-    <tableColumn id="30" xr3:uid="{32A00556-7442-4DB1-B296-A77DCB336CBB}" name="Aprovação concluída" dataDxfId="4"/>
-    <tableColumn id="31" xr3:uid="{8DFAFE87-22B8-4CBF-B231-61556BF451D2}" name="Aprovação Atrasada" dataDxfId="3"/>
-    <tableColumn id="32" xr3:uid="{F60F6277-6EE5-437A-B175-B8C884824A79}" name="Aderência" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{32358809-4D84-4EC6-9D6B-F35560F3DC76}" name="Id" dataDxfId="161"/>
+    <tableColumn id="2" xr3:uid="{FCB19FCF-87B1-4F17-A0AF-E2A9C7A37E14}" name="EDT" dataDxfId="160"/>
+    <tableColumn id="3" xr3:uid="{7B4C3492-A62F-4D65-BBF2-069B72009597}" name="Nome do Resumo da Tarefa" dataDxfId="159"/>
+    <tableColumn id="4" xr3:uid="{AD7B3DE1-9E98-459C-BDE3-9919792FF211}" name="Nome da Tarefa" dataDxfId="158"/>
+    <tableColumn id="5" xr3:uid="{92DFDBD7-E2BA-4076-951E-CF16C7ACC9C8}" name="Título" dataDxfId="157"/>
+    <tableColumn id="6" xr3:uid="{AC61FD1A-02A4-4608-AD57-A107FA721510}" name="Duração" dataDxfId="156"/>
+    <tableColumn id="7" xr3:uid="{9BE80CD5-26B0-4EB9-A979-0FC73B0DA5C1}" name="Início" dataDxfId="155"/>
+    <tableColumn id="8" xr3:uid="{C042A1D2-CD11-451A-BB2E-ADF748E717B7}" name="Término" dataDxfId="154"/>
+    <tableColumn id="9" xr3:uid="{34B72A3E-C902-4F09-A15E-BE98CDEBA5DC}" name="Predecessoras" dataDxfId="153"/>
+    <tableColumn id="10" xr3:uid="{31D2A1DA-CB2D-4FF9-804B-2BCF79701600}" name="% concluída" dataDxfId="152"/>
+    <tableColumn id="11" xr3:uid="{1C5DB045-C98A-41DA-A131-D34F37499306}" name="Término real" dataDxfId="151"/>
+    <tableColumn id="12" xr3:uid="{C5DBA407-4507-4B9D-A13E-CF0E5B37F4CB}" name="Status" dataDxfId="150"/>
+    <tableColumn id="13" xr3:uid="{7FD0F52D-F14B-4094-9B86-E31407658E6F}" name="Crítica" dataDxfId="149"/>
+    <tableColumn id="14" xr3:uid="{7C23A16E-8B3B-4CE8-AC03-22AC7CF72944}" name="Disciplina" dataDxfId="148"/>
+    <tableColumn id="15" xr3:uid="{88A23DF0-3034-4C7F-88CF-2DB38B1912FA}" name="Inicio_LB_R0" dataDxfId="147"/>
+    <tableColumn id="16" xr3:uid="{392A346F-3130-451B-A21F-E3796E7334D3}" name="Término_LB_R0" dataDxfId="146"/>
+    <tableColumn id="17" xr3:uid="{B9376082-58D3-49C9-A5B2-3C92CDBDEF3F}" name="Sprint" dataDxfId="145"/>
+    <tableColumn id="18" xr3:uid="{0CF4B4D4-ADC5-4588-B459-CC9363BB628A}" name="Sucessoras" dataDxfId="144"/>
+    <tableColumn id="19" xr3:uid="{DC3CD69F-D143-4C72-A08D-3F6B3D9E2249}" name="Comparação" dataDxfId="143"/>
+    <tableColumn id="20" xr3:uid="{945E3C0B-F472-404B-908F-FA76314CBA06}" name="Nomes dos recursos" dataDxfId="142"/>
+    <tableColumn id="21" xr3:uid="{E8B58DDB-65B5-4CA3-BC94-BC6B83061F33}" name="pct_val" dataDxfId="141"/>
+    <tableColumn id="22" xr3:uid="{082E8DFC-12B4-4EF3-BF47-3B3E6C3402E6}" name="Emissão inicial total" dataDxfId="140"/>
+    <tableColumn id="23" xr3:uid="{56C00BFF-1CD0-4CA8-84E4-E64001C6BED1}" name="Emissão inicial concluída" dataDxfId="139"/>
+    <tableColumn id="24" xr3:uid="{D2BA410D-4E72-405E-8AE7-050A5615443E}" name="Emissão Inicial Atrasada" dataDxfId="138"/>
+    <tableColumn id="25" xr3:uid="{675921B6-37F4-4A25-8D73-49B885233FFB}" name="Aprovação total" dataDxfId="137"/>
+    <tableColumn id="26" xr3:uid="{EACBFD06-8091-40A3-84B2-A054E3939CBE}" name="Avaliação do cliente concluída" dataDxfId="136"/>
+    <tableColumn id="27" xr3:uid="{FB495C50-A60D-4AA1-993F-9434537E0198}" name="Avaliação Cliente Atrasada" dataDxfId="135"/>
+    <tableColumn id="28" xr3:uid="{A73FCDFE-A256-4469-830F-FEED2901F101}" name="Atendimento de comentário concluído" dataDxfId="134"/>
+    <tableColumn id="29" xr3:uid="{79F7235A-C25E-4E99-8A10-F9E041C573F8}" name="Atendimento Atrasado" dataDxfId="133"/>
+    <tableColumn id="30" xr3:uid="{32A00556-7442-4DB1-B296-A77DCB336CBB}" name="Aprovação concluída" dataDxfId="132"/>
+    <tableColumn id="31" xr3:uid="{8DFAFE87-22B8-4CBF-B231-61556BF451D2}" name="Aprovação Atrasada" dataDxfId="131"/>
+    <tableColumn id="32" xr3:uid="{F60F6277-6EE5-437A-B175-B8C884824A79}" name="Aderência" dataDxfId="130"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{7E4114E9-02FF-411C-95F0-16D1DC253DF8}" name="Tabela7" displayName="Tabela7" ref="A1:K75" totalsRowShown="0" headerRowDxfId="2" dataDxfId="1">
+  <autoFilter ref="A1:K75" xr:uid="{7E4114E9-02FF-411C-95F0-16D1DC253DF8}">
+    <filterColumn colId="4">
+      <filters>
+        <filter val="emissão inicial"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{A831729F-5781-4E64-B2B6-BA8E9E5324C9}" name="Sprint" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{54BD9B53-2427-4A5D-8FD3-5CCC7CDBFC96}" name="Id" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{6980DA4C-6748-4512-B658-9BDA0901D8AB}" name="EDT" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{ECC3F254-5B80-4623-8054-764293517B3D}" name="Nome do Resumo da Tarefa" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{B9D73B8A-A72F-43D5-A7AA-E10F483188C4}" name="Nome da Tarefa" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{5E25BE0A-86F5-4D1D-8252-510C0899C7CF}" name="Status" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{D998A76A-DD65-42FC-AB7F-5C195E733E5D}" name="% concluída" dataDxfId="6" dataCellStyle="Porcentagem"/>
+    <tableColumn id="8" xr3:uid="{B8081E71-0AFF-4C40-BEC6-91FD4975EC84}" name="Nomes dos recursos" dataDxfId="5"/>
+    <tableColumn id="9" xr3:uid="{57C285FE-48AE-448B-9F62-E1A0753BA64A}" name="Disciplina" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{CEC8088D-5182-489C-B327-9855A66A3881}" name="Crítica" dataDxfId="3"/>
+    <tableColumn id="11" xr3:uid="{CC40F17F-3187-4201-B5E1-B0F44823548F}" name="Coluna1" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -35616,7 +35136,7 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="B17" s="1">
         <f>SUBTOTAL(109,Tabela1[Emissão inicial total])</f>
@@ -35881,7 +35401,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="B36" s="1">
         <f>SUBTOTAL(109,Tabela2[Emissão Inicial Atrasada])</f>
@@ -35926,7 +35446,7 @@
     <col min="15" max="16384" width="13" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>454</v>
       </c>
@@ -44131,6 +43651,22 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="iconSet" priority="1" id="{03AF946E-5AC7-4E9C-BEF6-465FA50619D5}">
+            <x14:iconSet iconSet="3Triangles">
+              <x14:cfvo type="percent">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="percent">
+                <xm:f>33</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="percent">
+                <xm:f>67</xm:f>
+              </x14:cfvo>
+            </x14:iconSet>
+          </x14:cfRule>
+          <xm:sqref>L1:L187</xm:sqref>
+        </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="iconSet" priority="2" id="{F7CE81E8-3D3D-4082-9138-58DEE688B6F2}">
             <x14:iconSet iconSet="3Triangles">
@@ -44146,22 +43682,6 @@
             </x14:iconSet>
           </x14:cfRule>
           <xm:sqref>O1:O187</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="iconSet" priority="1" id="{03AF946E-5AC7-4E9C-BEF6-465FA50619D5}">
-            <x14:iconSet iconSet="3Triangles">
-              <x14:cfvo type="percent">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="percent">
-                <xm:f>33</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="percent">
-                <xm:f>67</xm:f>
-              </x14:cfvo>
-            </x14:iconSet>
-          </x14:cfRule>
-          <xm:sqref>L1:L187</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -51252,2177 +50772,2234 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:J75"/>
+  <dimension ref="A1:K75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="32.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="K1" s="1" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="1">
         <v>1</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="1">
         <v>1</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="4">
         <v>0.28999999999999998</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="1">
         <v>2</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="4">
         <v>0.28999999999999998</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="1">
         <v>6</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="4">
         <v>0.79</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="1">
         <v>7</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="4">
         <v>0.7</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="1">
         <v>12</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="4">
         <v>0.81</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="J6" t="s">
+      <c r="J6" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="1">
         <v>15</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="4">
         <v>0.5</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="J7" t="s">
+      <c r="J7" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="1">
         <v>16</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="I8" t="s">
+      <c r="G8" s="4">
+        <v>0</v>
+      </c>
+      <c r="I8" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="J8" t="s">
+      <c r="J8" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="1">
         <v>17</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="4">
         <v>0.81</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I9" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="J9" t="s">
+      <c r="J9" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="1">
         <v>20</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="4">
         <v>0.5</v>
       </c>
-      <c r="I10" t="s">
+      <c r="I10" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="J10" t="s">
+      <c r="J10" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="1">
         <v>21</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G11">
-        <v>0</v>
-      </c>
-      <c r="I11" t="s">
+      <c r="G11" s="4">
+        <v>0</v>
+      </c>
+      <c r="I11" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="J11" t="s">
+      <c r="J11" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="1">
         <v>22</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="4">
         <v>0.4</v>
       </c>
-      <c r="I12" t="s">
+      <c r="I12" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J12" t="s">
+      <c r="J12" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="1">
         <v>23</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G13">
-        <v>0</v>
-      </c>
-      <c r="I13" t="s">
+      <c r="G13" s="4">
+        <v>0</v>
+      </c>
+      <c r="I13" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J13" t="s">
+      <c r="J13" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="1">
         <v>24</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G14">
-        <v>0</v>
-      </c>
-      <c r="I14" t="s">
+      <c r="G14" s="4">
+        <v>0</v>
+      </c>
+      <c r="I14" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J14" t="s">
+      <c r="J14" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="1">
         <v>25</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G15">
-        <v>0</v>
-      </c>
-      <c r="I15" t="s">
+      <c r="G15" s="4">
+        <v>0</v>
+      </c>
+      <c r="I15" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J15" t="s">
+      <c r="J15" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="1">
         <v>26</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G16">
-        <v>0</v>
-      </c>
-      <c r="I16" t="s">
+      <c r="G16" s="4">
+        <v>0</v>
+      </c>
+      <c r="I16" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J16" t="s">
+      <c r="J16" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="17" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="1">
         <v>27</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G17">
-        <v>0</v>
-      </c>
-      <c r="I17" t="s">
+      <c r="G17" s="4">
+        <v>0</v>
+      </c>
+      <c r="I17" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J17" t="s">
+      <c r="J17" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="1">
         <v>28</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G18">
-        <v>0</v>
-      </c>
-      <c r="I18" t="s">
+      <c r="G18" s="4">
+        <v>0</v>
+      </c>
+      <c r="I18" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J18" t="s">
+      <c r="J18" s="1" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B19">
+      <c r="B19" s="1">
         <v>29</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G19">
-        <v>0</v>
-      </c>
-      <c r="I19" t="s">
+      <c r="G19" s="4">
+        <v>0</v>
+      </c>
+      <c r="I19" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J19" t="s">
+      <c r="J19" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B20">
+    <row r="20" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="1">
         <v>30</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G20">
-        <v>0</v>
-      </c>
-      <c r="I20" t="s">
+      <c r="G20" s="4">
+        <v>0</v>
+      </c>
+      <c r="I20" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J20" t="s">
+      <c r="J20" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B21">
+    <row r="21" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="1">
         <v>31</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G21">
-        <v>0</v>
-      </c>
-      <c r="I21" t="s">
+      <c r="G21" s="4">
+        <v>0</v>
+      </c>
+      <c r="I21" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J21" t="s">
+      <c r="J21" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B22">
+    <row r="22" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="1">
         <v>32</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G22">
-        <v>0</v>
-      </c>
-      <c r="I22" t="s">
+      <c r="G22" s="4">
+        <v>0</v>
+      </c>
+      <c r="I22" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J22" t="s">
+      <c r="J22" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="23" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="1">
         <v>33</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="4">
         <v>0.71</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J23" t="s">
+      <c r="J23" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="24" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="1">
         <v>36</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F24" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G24">
+      <c r="G24" s="4">
         <v>0.5</v>
       </c>
-      <c r="I24" t="s">
+      <c r="I24" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J24" t="s">
+      <c r="J24" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="25" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="1">
         <v>37</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G25">
-        <v>0</v>
-      </c>
-      <c r="I25" t="s">
+      <c r="G25" s="4">
+        <v>0</v>
+      </c>
+      <c r="I25" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J25" t="s">
+      <c r="J25" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="26" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="1">
         <v>38</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F26" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G26">
+      <c r="G26" s="4">
         <v>0.71</v>
       </c>
-      <c r="I26" t="s">
+      <c r="I26" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J26" t="s">
+      <c r="J26" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="27" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="1">
         <v>43</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G27">
+      <c r="G27" s="4">
         <v>0.31</v>
       </c>
-      <c r="I27" t="s">
+      <c r="I27" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="J27" t="s">
+      <c r="J27" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="28" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B28">
+      <c r="B28" s="1">
         <v>44</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E28" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F28" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G28">
+      <c r="G28" s="4">
         <v>0.28000000000000003</v>
       </c>
-      <c r="I28" t="s">
+      <c r="I28" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="J28" t="s">
+      <c r="J28" s="1" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+      <c r="A29" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B29">
+      <c r="B29" s="1">
         <v>45</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E29" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F29" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G29">
+      <c r="G29" s="4">
         <v>0.5</v>
       </c>
-      <c r="I29" t="s">
+      <c r="I29" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="J29" t="s">
+      <c r="J29" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="30" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B30">
+      <c r="B30" s="1">
         <v>46</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F30" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G30">
-        <v>0</v>
-      </c>
-      <c r="I30" t="s">
+      <c r="G30" s="4">
+        <v>0</v>
+      </c>
+      <c r="I30" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="J30" t="s">
+      <c r="J30" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row r="31" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B31">
+      <c r="B31" s="1">
         <v>47</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F31" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G31">
-        <v>0</v>
-      </c>
-      <c r="I31" t="s">
+      <c r="G31" s="4">
+        <v>0</v>
+      </c>
+      <c r="I31" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="J31" t="s">
+      <c r="J31" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row r="32" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B32">
+      <c r="B32" s="1">
         <v>48</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E32" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F32" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G32">
-        <v>0</v>
-      </c>
-      <c r="I32" t="s">
+      <c r="G32" s="4">
+        <v>0</v>
+      </c>
+      <c r="I32" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="J32" t="s">
+      <c r="J32" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="33" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B33">
+      <c r="B33" s="1">
         <v>54</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D33" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E33" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="F33" t="s">
+      <c r="F33" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G33">
+      <c r="G33" s="4">
         <v>0.63</v>
       </c>
-      <c r="I33" t="s">
+      <c r="I33" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="J33" t="s">
+      <c r="J33" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+    <row r="34" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B34">
+      <c r="B34" s="1">
         <v>57</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C34" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D34" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="E34" t="s">
+      <c r="E34" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F34" t="s">
+      <c r="F34" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G34">
+      <c r="G34" s="4">
         <v>0.75</v>
       </c>
-      <c r="I34" t="s">
+      <c r="I34" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="J34" t="s">
+      <c r="J34" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+    <row r="35" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B35">
+      <c r="B35" s="1">
         <v>58</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C35" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D35" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="E35" t="s">
+      <c r="E35" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F35" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G35">
-        <v>0</v>
-      </c>
-      <c r="I35" t="s">
+      <c r="G35" s="4">
+        <v>0</v>
+      </c>
+      <c r="I35" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="J35" t="s">
+      <c r="J35" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    <row r="36" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B36">
+      <c r="B36" s="1">
         <v>59</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C36" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D36" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="E36" t="s">
+      <c r="E36" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="F36" t="s">
+      <c r="F36" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G36">
+      <c r="G36" s="4">
         <v>0.63</v>
       </c>
-      <c r="I36" t="s">
+      <c r="I36" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="J36" t="s">
+      <c r="J36" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+    <row r="37" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B37">
+      <c r="B37" s="1">
         <v>62</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C37" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D37" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="E37" t="s">
+      <c r="E37" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F37" t="s">
+      <c r="F37" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G37">
+      <c r="G37" s="4">
         <v>0.75</v>
       </c>
-      <c r="I37" t="s">
+      <c r="I37" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="J37" t="s">
+      <c r="J37" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+    <row r="38" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B38">
+      <c r="B38" s="1">
         <v>63</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C38" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D38" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="E38" t="s">
+      <c r="E38" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="F38" t="s">
+      <c r="F38" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G38">
-        <v>0</v>
-      </c>
-      <c r="I38" t="s">
+      <c r="G38" s="4">
+        <v>0</v>
+      </c>
+      <c r="I38" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="J38" t="s">
+      <c r="J38" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+    <row r="39" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B39">
+      <c r="B39" s="1">
         <v>64</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C39" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D39" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E39" t="s">
+      <c r="E39" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="F39" t="s">
+      <c r="F39" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G39">
+      <c r="G39" s="4">
         <v>0.09</v>
       </c>
-      <c r="I39" t="s">
+      <c r="I39" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="J39" t="s">
+      <c r="J39" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+    <row r="40" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B40">
+      <c r="B40" s="1">
         <v>65</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C40" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D40" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="E40" t="s">
+      <c r="E40" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="F40" t="s">
+      <c r="F40" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G40">
+      <c r="G40" s="4">
         <v>0.67</v>
       </c>
-      <c r="I40" t="s">
+      <c r="I40" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="J40" t="s">
+      <c r="J40" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+    <row r="41" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B41">
+      <c r="B41" s="1">
         <v>68</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C41" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D41" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="E41" t="s">
+      <c r="E41" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F41" t="s">
+      <c r="F41" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G41">
+      <c r="G41" s="4">
         <v>0.5</v>
       </c>
-      <c r="I41" t="s">
+      <c r="I41" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="J41" t="s">
+      <c r="J41" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+    <row r="42" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B42">
+      <c r="B42" s="1">
         <v>69</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C42" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="D42" t="s">
+      <c r="D42" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="E42" t="s">
+      <c r="E42" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="F42" t="s">
+      <c r="F42" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G42">
-        <v>0</v>
-      </c>
-      <c r="I42" t="s">
+      <c r="G42" s="4">
+        <v>0</v>
+      </c>
+      <c r="I42" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="J42" t="s">
+      <c r="J42" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+    <row r="43" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B43">
+      <c r="B43" s="1">
         <v>95</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C43" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="D43" t="s">
+      <c r="D43" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="E43" t="s">
+      <c r="E43" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="F43" t="s">
+      <c r="F43" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G43">
-        <v>0</v>
-      </c>
-      <c r="I43" t="s">
+      <c r="G43" s="4">
+        <v>0</v>
+      </c>
+      <c r="I43" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="J43" t="s">
+      <c r="J43" s="1" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+      <c r="A44" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B44">
+      <c r="B44" s="1">
         <v>96</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C44" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="D44" t="s">
+      <c r="D44" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="E44" t="s">
+      <c r="E44" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="F44" t="s">
+      <c r="F44" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G44">
-        <v>0</v>
-      </c>
-      <c r="I44" t="s">
+      <c r="G44" s="4">
+        <v>0</v>
+      </c>
+      <c r="I44" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="J44" t="s">
+      <c r="J44" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+    <row r="45" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B45">
+      <c r="B45" s="1">
         <v>100</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C45" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="D45" t="s">
+      <c r="D45" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E45" t="s">
+      <c r="E45" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="F45" t="s">
+      <c r="F45" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G45">
+      <c r="G45" s="4">
         <v>0.39</v>
       </c>
-      <c r="I45" t="s">
+      <c r="I45" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="J45" t="s">
+      <c r="J45" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+    <row r="46" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B46">
+      <c r="B46" s="1">
         <v>111</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C46" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="D46" t="s">
+      <c r="D46" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="E46" t="s">
+      <c r="E46" s="1" t="s">
         <v>310</v>
       </c>
-      <c r="F46" t="s">
+      <c r="F46" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G46">
-        <v>0</v>
-      </c>
-      <c r="I46" t="s">
+      <c r="G46" s="4">
+        <v>0</v>
+      </c>
+      <c r="I46" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="J46" t="s">
+      <c r="J46" s="1" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+      <c r="A47" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B47">
+      <c r="B47" s="1">
         <v>112</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C47" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="D47" t="s">
+      <c r="D47" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="E47" t="s">
+      <c r="E47" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="F47" t="s">
+      <c r="F47" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G47">
-        <v>0</v>
-      </c>
-      <c r="I47" t="s">
+      <c r="G47" s="4">
+        <v>0</v>
+      </c>
+      <c r="I47" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="J47" t="s">
+      <c r="J47" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
+    <row r="48" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B48">
+      <c r="B48" s="1">
         <v>116</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C48" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="D48" t="s">
+      <c r="D48" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E48" t="s">
+      <c r="E48" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="F48" t="s">
+      <c r="F48" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G48">
+      <c r="G48" s="4">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="I48" t="s">
+      <c r="I48" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="J48" t="s">
+      <c r="J48" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
+    <row r="49" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B49">
+      <c r="B49" s="1">
         <v>117</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C49" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="D49" t="s">
+      <c r="D49" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="E49" t="s">
+      <c r="E49" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="F49" t="s">
+      <c r="F49" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G49">
+      <c r="G49" s="4">
         <v>0.21</v>
       </c>
-      <c r="I49" t="s">
+      <c r="I49" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="J49" t="s">
+      <c r="J49" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B50">
+      <c r="B50" s="1">
         <v>118</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C50" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="D50" t="s">
+      <c r="D50" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="E50" t="s">
+      <c r="E50" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="F50" t="s">
+      <c r="F50" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G50">
+      <c r="G50" s="4">
         <v>0.5</v>
       </c>
-      <c r="I50" t="s">
+      <c r="I50" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="J50" t="s">
+      <c r="J50" s="1" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
+      <c r="K50" s="14">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B51">
+      <c r="B51" s="1">
         <v>119</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C51" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="D51" t="s">
+      <c r="D51" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="E51" t="s">
+      <c r="E51" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F51" t="s">
+      <c r="F51" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G51">
-        <v>0</v>
-      </c>
-      <c r="I51" t="s">
+      <c r="G51" s="4">
+        <v>0</v>
+      </c>
+      <c r="I51" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="J51" t="s">
+      <c r="J51" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
+    <row r="52" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B52">
+      <c r="B52" s="1">
         <v>120</v>
       </c>
-      <c r="C52" t="s">
+      <c r="C52" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="D52" t="s">
+      <c r="D52" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="E52" t="s">
+      <c r="E52" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F52" t="s">
+      <c r="F52" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G52">
-        <v>0</v>
-      </c>
-      <c r="I52" t="s">
+      <c r="G52" s="4">
+        <v>0</v>
+      </c>
+      <c r="I52" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="J52" t="s">
+      <c r="J52" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
+    <row r="53" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B53">
+      <c r="B53" s="1">
         <v>121</v>
       </c>
-      <c r="C53" t="s">
+      <c r="C53" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="D53" t="s">
+      <c r="D53" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="E53" t="s">
+      <c r="E53" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="F53" t="s">
+      <c r="F53" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G53">
-        <v>0</v>
-      </c>
-      <c r="I53" t="s">
+      <c r="G53" s="4">
+        <v>0</v>
+      </c>
+      <c r="I53" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="J53" t="s">
+      <c r="J53" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
+    <row r="54" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B54">
+      <c r="B54" s="1">
         <v>127</v>
       </c>
-      <c r="C54" t="s">
+      <c r="C54" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="D54" t="s">
+      <c r="D54" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="E54" t="s">
+      <c r="E54" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="F54" t="s">
+      <c r="F54" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G54">
-        <v>0</v>
-      </c>
-      <c r="I54" t="s">
+      <c r="G54" s="4">
+        <v>0</v>
+      </c>
+      <c r="I54" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="J54" t="s">
+      <c r="J54" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A55" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B55">
+      <c r="B55" s="1">
         <v>128</v>
       </c>
-      <c r="C55" t="s">
+      <c r="C55" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="D55" t="s">
+      <c r="D55" s="1" t="s">
         <v>343</v>
       </c>
-      <c r="E55" t="s">
+      <c r="E55" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="F55" t="s">
+      <c r="F55" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G55">
-        <v>0</v>
-      </c>
-      <c r="I55" t="s">
+      <c r="G55" s="4">
+        <v>0</v>
+      </c>
+      <c r="I55" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="J55" t="s">
+      <c r="J55" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
+    <row r="56" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B56">
+      <c r="B56" s="1">
         <v>132</v>
       </c>
-      <c r="C56" t="s">
+      <c r="C56" s="1" t="s">
         <v>347</v>
       </c>
-      <c r="D56" t="s">
+      <c r="D56" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E56" t="s">
+      <c r="E56" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="F56" t="s">
+      <c r="F56" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G56">
+      <c r="G56" s="4">
         <v>0.28999999999999998</v>
       </c>
-      <c r="I56" t="s">
+      <c r="I56" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="J56" t="s">
+      <c r="J56" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
+    <row r="57" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B57">
+      <c r="B57" s="1">
         <v>133</v>
       </c>
-      <c r="C57" t="s">
+      <c r="C57" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="D57" t="s">
+      <c r="D57" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="E57" t="s">
+      <c r="E57" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="F57" t="s">
+      <c r="F57" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G57">
+      <c r="G57" s="4">
         <v>0.8</v>
       </c>
-      <c r="I57" t="s">
+      <c r="I57" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="J57" t="s">
+      <c r="J57" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
+    <row r="58" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B58">
+      <c r="B58" s="1">
         <v>136</v>
       </c>
-      <c r="C58" t="s">
+      <c r="C58" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="D58" t="s">
+      <c r="D58" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="E58" t="s">
+      <c r="E58" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F58" t="s">
+      <c r="F58" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G58">
+      <c r="G58" s="4">
         <v>0.5</v>
       </c>
-      <c r="I58" t="s">
+      <c r="I58" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="J58" t="s">
+      <c r="J58" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
+    <row r="59" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B59">
+      <c r="B59" s="1">
         <v>137</v>
       </c>
-      <c r="C59" t="s">
+      <c r="C59" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="D59" t="s">
+      <c r="D59" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="E59" t="s">
+      <c r="E59" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="F59" t="s">
+      <c r="F59" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G59">
-        <v>0</v>
-      </c>
-      <c r="I59" t="s">
+      <c r="G59" s="4">
+        <v>0</v>
+      </c>
+      <c r="I59" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="J59" t="s">
+      <c r="J59" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
+    <row r="60" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B60">
+      <c r="B60" s="1">
         <v>143</v>
       </c>
-      <c r="C60" t="s">
+      <c r="C60" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="D60" t="s">
+      <c r="D60" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="E60" t="s">
+      <c r="E60" s="1" t="s">
         <v>371</v>
       </c>
-      <c r="F60" t="s">
+      <c r="F60" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G60">
-        <v>0</v>
-      </c>
-      <c r="I60" t="s">
+      <c r="G60" s="4">
+        <v>0</v>
+      </c>
+      <c r="I60" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="J60" t="s">
+      <c r="J60" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A61" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B61">
+      <c r="B61" s="1">
         <v>144</v>
       </c>
-      <c r="C61" t="s">
+      <c r="C61" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="D61" t="s">
+      <c r="D61" s="1" t="s">
         <v>373</v>
       </c>
-      <c r="E61" t="s">
+      <c r="E61" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="F61" t="s">
+      <c r="F61" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G61">
-        <v>0</v>
-      </c>
-      <c r="I61" t="s">
+      <c r="G61" s="4">
+        <v>0</v>
+      </c>
+      <c r="I61" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="J61" t="s">
+      <c r="J61" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
+    <row r="62" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B62">
+      <c r="B62" s="1">
         <v>148</v>
       </c>
-      <c r="C62" t="s">
+      <c r="C62" s="1" t="s">
         <v>377</v>
       </c>
-      <c r="D62" t="s">
+      <c r="D62" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E62" t="s">
+      <c r="E62" s="1" t="s">
         <v>378</v>
       </c>
-      <c r="F62" t="s">
+      <c r="F62" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G62">
+      <c r="G62" s="4">
         <v>0.23</v>
       </c>
-      <c r="I62" t="s">
+      <c r="I62" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="J62" t="s">
+      <c r="J62" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
+    <row r="63" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B63">
+      <c r="B63" s="1">
         <v>149</v>
       </c>
-      <c r="C63" t="s">
+      <c r="C63" s="1" t="s">
         <v>381</v>
       </c>
-      <c r="D63" t="s">
+      <c r="D63" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="E63" t="s">
+      <c r="E63" s="1" t="s">
         <v>383</v>
       </c>
-      <c r="F63" t="s">
+      <c r="F63" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G63">
+      <c r="G63" s="4">
         <v>0.5</v>
       </c>
-      <c r="I63" t="s">
+      <c r="I63" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="J63" t="s">
+      <c r="J63" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
+    <row r="64" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B64">
+      <c r="B64" s="1">
         <v>152</v>
       </c>
-      <c r="C64" t="s">
+      <c r="C64" s="1" t="s">
         <v>388</v>
       </c>
-      <c r="D64" t="s">
+      <c r="D64" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="E64" t="s">
+      <c r="E64" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F64" t="s">
+      <c r="F64" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G64">
+      <c r="G64" s="4">
         <v>0.5</v>
       </c>
-      <c r="I64" t="s">
+      <c r="I64" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="J64" t="s">
+      <c r="J64" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
+    <row r="65" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B65">
+      <c r="B65" s="1">
         <v>153</v>
       </c>
-      <c r="C65" t="s">
+      <c r="C65" s="1" t="s">
         <v>389</v>
       </c>
-      <c r="D65" t="s">
+      <c r="D65" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="E65" t="s">
+      <c r="E65" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="F65" t="s">
+      <c r="F65" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G65">
-        <v>0</v>
-      </c>
-      <c r="I65" t="s">
+      <c r="G65" s="4">
+        <v>0</v>
+      </c>
+      <c r="I65" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="J65" t="s">
+      <c r="J65" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
+    <row r="66" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B66">
+      <c r="B66" s="1">
         <v>154</v>
       </c>
-      <c r="C66" t="s">
+      <c r="C66" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="D66" t="s">
+      <c r="D66" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="E66" t="s">
+      <c r="E66" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="F66" t="s">
+      <c r="F66" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G66">
+      <c r="G66" s="4">
         <v>0.5</v>
       </c>
-      <c r="I66" t="s">
+      <c r="I66" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="J66" t="s">
+      <c r="J66" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
+    <row r="67" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B67">
+      <c r="B67" s="1">
         <v>157</v>
       </c>
-      <c r="C67" t="s">
+      <c r="C67" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="D67" t="s">
+      <c r="D67" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="E67" t="s">
+      <c r="E67" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F67" t="s">
+      <c r="F67" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G67">
+      <c r="G67" s="4">
         <v>0.5</v>
       </c>
-      <c r="I67" t="s">
+      <c r="I67" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="J67" t="s">
+      <c r="J67" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
+    <row r="68" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B68">
+      <c r="B68" s="1">
         <v>158</v>
       </c>
-      <c r="C68" t="s">
+      <c r="C68" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="D68" t="s">
+      <c r="D68" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="E68" t="s">
+      <c r="E68" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="F68" t="s">
+      <c r="F68" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G68">
-        <v>0</v>
-      </c>
-      <c r="I68" t="s">
+      <c r="G68" s="4">
+        <v>0</v>
+      </c>
+      <c r="I68" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="J68" t="s">
+      <c r="J68" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
+    <row r="69" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B69">
+      <c r="B69" s="1">
         <v>164</v>
       </c>
-      <c r="C69" t="s">
+      <c r="C69" s="1" t="s">
         <v>409</v>
       </c>
-      <c r="D69" t="s">
+      <c r="D69" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="E69" t="s">
+      <c r="E69" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="F69" t="s">
+      <c r="F69" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G69">
-        <v>0</v>
-      </c>
-      <c r="I69" t="s">
+      <c r="G69" s="4">
+        <v>0</v>
+      </c>
+      <c r="I69" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="J69" t="s">
+      <c r="J69" s="1" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
+      <c r="A70" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B70">
+      <c r="B70" s="1">
         <v>165</v>
       </c>
-      <c r="C70" t="s">
+      <c r="C70" s="1" t="s">
         <v>411</v>
       </c>
-      <c r="D70" t="s">
+      <c r="D70" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="E70" t="s">
+      <c r="E70" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="F70" t="s">
+      <c r="F70" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G70">
-        <v>0</v>
-      </c>
-      <c r="I70" t="s">
+      <c r="G70" s="4">
+        <v>0</v>
+      </c>
+      <c r="I70" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="J70" t="s">
+      <c r="J70" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
+    <row r="71" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B71">
+      <c r="B71" s="1">
         <v>169</v>
       </c>
-      <c r="C71" t="s">
+      <c r="C71" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="D71" t="s">
+      <c r="D71" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="E71" t="s">
+      <c r="E71" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="F71" t="s">
+      <c r="F71" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G71">
+      <c r="G71" s="4">
         <v>0.39</v>
       </c>
-      <c r="I71" t="s">
+      <c r="I71" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="J71" t="s">
+      <c r="J71" s="1" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
+      <c r="A72" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B72">
+      <c r="B72" s="12">
         <v>170</v>
       </c>
-      <c r="C72" t="s">
+      <c r="C72" s="12" t="s">
         <v>418</v>
       </c>
-      <c r="D72" t="s">
+      <c r="D72" s="12" t="s">
         <v>419</v>
       </c>
-      <c r="E72" t="s">
+      <c r="E72" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="F72" t="s">
+      <c r="F72" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="G72">
-        <v>0.9</v>
-      </c>
-      <c r="I72" t="s">
+      <c r="G72" s="13">
+        <v>1</v>
+      </c>
+      <c r="H72" s="12"/>
+      <c r="I72" s="12" t="s">
         <v>380</v>
       </c>
-      <c r="J72" t="s">
+      <c r="J72" s="12" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+    <row r="73" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B73">
+      <c r="B73" s="1">
         <v>171</v>
       </c>
-      <c r="C73" t="s">
+      <c r="C73" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="D73" t="s">
+      <c r="D73" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="E73" t="s">
+      <c r="E73" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F73" t="s">
+      <c r="F73" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="G73">
-        <v>0</v>
-      </c>
-      <c r="I73" t="s">
+      <c r="G73" s="4">
+        <v>0</v>
+      </c>
+      <c r="I73" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="J73" t="s">
+      <c r="J73" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
+    <row r="74" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B74">
+      <c r="B74" s="1">
         <v>172</v>
       </c>
-      <c r="C74" t="s">
+      <c r="C74" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="D74" t="s">
+      <c r="D74" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="E74" t="s">
+      <c r="E74" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F74" t="s">
+      <c r="F74" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="G74">
-        <v>0</v>
-      </c>
-      <c r="I74" t="s">
+      <c r="G74" s="4">
+        <v>0</v>
+      </c>
+      <c r="I74" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="J74" t="s">
+      <c r="J74" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
+    <row r="75" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B75">
+      <c r="B75" s="1">
         <v>7</v>
       </c>
-      <c r="C75" t="s">
+      <c r="C75" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D75" t="s">
+      <c r="D75" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E75" t="s">
+      <c r="E75" s="1" t="s">
         <v>440</v>
       </c>
-      <c r="F75" t="s">
+      <c r="F75" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="G75">
-        <v>0</v>
-      </c>
-      <c r="I75" t="s">
+      <c r="G75" s="4">
+        <v>0</v>
+      </c>
+      <c r="I75" s="1" t="s">
         <v>442</v>
       </c>
-      <c r="J75" t="s">
+      <c r="J75" s="1" t="s">
         <v>35</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="G1:G1048576">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF008AEF"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{4FCABA3C-F2B7-4179-A16C-DE1702F74A09}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;11&amp;K000000 BV_C2_Internal</oddFooter>
   </headerFooter>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{4FCABA3C-F2B7-4179-A16C-DE1702F74A09}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF008AEF"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>G1:G1048576</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
@@ -53965,6 +53542,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c6385d03-c98b-47a8-b084-660309c480c9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="1dad954f-e29e-48a7-b9b8-f0523de1045f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B05075DB2EB95E4AB0084D2AB051A38A" ma:contentTypeVersion="10" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="1acf5709253336bc12ea482482f5d520">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c6385d03-c98b-47a8-b084-660309c480c9" xmlns:ns3="1dad954f-e29e-48a7-b9b8-f0523de1045f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="84ff94f6b93240dc82e76730a418228e" ns2:_="" ns3:_="">
     <xsd:import namespace="c6385d03-c98b-47a8-b084-660309c480c9"/>
@@ -54153,27 +53750,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24ACE1AF-9695-485E-AC7F-CBB0B2981F41}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c6385d03-c98b-47a8-b084-660309c480c9"/>
+    <ds:schemaRef ds:uri="1dad954f-e29e-48a7-b9b8-f0523de1045f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c6385d03-c98b-47a8-b084-660309c480c9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="1dad954f-e29e-48a7-b9b8-f0523de1045f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8138B1AB-1972-4DFF-B096-6552737E50BB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3EF5282B-EB3A-4047-A7AA-7FD92B2BC98F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -54190,23 +53786,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8138B1AB-1972-4DFF-B096-6552737E50BB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24ACE1AF-9695-485E-AC7F-CBB0B2981F41}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c6385d03-c98b-47a8-b084-660309c480c9"/>
-    <ds:schemaRef ds:uri="1dad954f-e29e-48a7-b9b8-f0523de1045f"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>